<commit_message>
PlayerBaseStat , WeaponData 수정
PlayerBaseStat에 MaxMana , ManaRegen 필드 추가
WeaponaData 에 WeaponReqMana , ManaPerAmmo 필드 추가
</commit_message>
<xml_diff>
--- a/Content/Data/PlayerBaseStat.xlsx
+++ b/Content/Data/PlayerBaseStat.xlsx
@@ -460,13 +460,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,6 +490,21 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>MaxMana</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ManaRegen</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>JumpPower</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Comment</t>
         </is>
       </c>
@@ -509,6 +527,21 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>[int]</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[float]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>[float]</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>[string]</t>
         </is>
       </c>
@@ -530,6 +563,21 @@
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>최대 마나</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>초당 마나 회복량</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>점프력</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>기획 메모(변환시 제외)</t>
         </is>
@@ -545,14 +593,23 @@
       <c r="C4" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>420</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>기본 스탯</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="6">
     <dataValidation sqref="A4:A500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="범위 오류" error="Hp는 0보다 커야 합니다." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
@@ -560,6 +617,15 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="C4:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="범위 오류" error="RunSpeed는 0보다 커야 합니다." type="decimal" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="범위 오류" error="MaxMana는 0보다 커야 합니다." type="decimal" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="범위 오류" error="ManaRegen는 0보다 커야 합니다." type="decimal" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="범위 오류" error="JumpPower는 0보다 커야 합니다." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
발사모드(Single/FullAuto/Burst)·HP/Mana 회복·ADS 조준 시스템 추가
- MainWeaponComponent: FireMode(Single/FullAuto/Burst) 실제 구현
  - FullAuto는 클라이언트 반복 타이머, Burst는 서버 타이머로 나머지 탄 처리(매 탄마다 실시간 조준 방향 재조회)
  - EquipWeapon() 무기 교체 시 이전 무기의 FullAuto/Burst 타이머 정리, WeaponIndex 복제 및 OnRep로 클라이언트 재로드
  - StartADS/StopADS/Server_SetAiming으로 조준 상태 추가, GetADSSpeed() 노출
  - 클라이언트에서도 EquipWeapon()이 실행되도록 BeginPlay의 HasAuthority 제한 제거 (weapons.json 로컬 로딩)
  - GetWorld() null 체크 누락으로 인한 StopFire() 크래시 수정
- MainHPComponent/MainManaComponent: MainEffectTickComponent 신설
  - 주기적 회복 신호(OnEffectTick)를 별도 컴포넌트가 브로드캐스트, HP/Mana가 각자 구독해서 반응
  - HP는 HPRegen/HPRegenDelay(피격 후 회복 재개 지연) 반영, PlayerBaseStat.h의 MaxHP 필드명 변경 반영
- WeaponDataManager: static 멤버 정의 누락으로 인한 LNK2001 링크 에러 및 PIE 멀티플레이어 콘솔 명령어 중복 등록 크래시 수정
- BP_MainCharacter: 1인칭 카메라/무기 뷰모델(FirstPersonCamera, FirstPersonMesh) 및 ADS 시 조준경 정렬 연출 추가
- MainHUDWidget 신규: 본인 Hp/Mana/Ammo 표시 HUD, 사망 시 자동 제거
</commit_message>
<xml_diff>
--- a/Content/Data/PlayerBaseStat.xlsx
+++ b/Content/Data/PlayerBaseStat.xlsx
@@ -524,7 +524,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>[int]</t>
+          <t>[float]</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[int]</t>
+          <t>[float]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">

</xml_diff>